<commit_message>
Reports as of 2026-10-14 (main@b97528c)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-13. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-15 (main@341915a)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-14. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-16 (main@6e6b126)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-15. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-17 (main@6e6b126)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-16. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-18 (main@6e6b126)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-17. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-19 (main@2597efb)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-18. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-20 (main@2597efb)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-19. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-21 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-20. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-22 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-21. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-23 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-22. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-24 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-23. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-25 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-24. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-26 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-25. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-27 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-26. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-28 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-27. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-29 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-28. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-30 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-29. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reports as of 2026-10-31 (main@83ac175)
</commit_message>
<xml_diff>
--- a/example-client-iso42001-workbook.xlsx
+++ b/example-client-iso42001-workbook.xlsx
@@ -571,7 +571,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -4991,7 +4991,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -6441,7 +6441,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7232,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8385,7 +8385,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -8764,7 +8764,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>
@@ -9551,7 +9551,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-30. Read-only export: change the record through pull requests, not here.</t>
+          <t>(Example Client) · ISO 42001 · generated from the GRC record as of 2026-10-31. Read-only export: change the record through pull requests, not here.</t>
         </is>
       </c>
     </row>

</xml_diff>